<commit_message>
Hito H3: los dos agentes navegan a la vez, cada uno en su piso
0,281 m y 0,143 m de error real contra /odom. El control es robot2 solo el
24-ago, que dio 0,190 m: con otro agente corriendo no empeora.

El /odom cruzado que bloqueaba el hito se cierra con causa y no por no
reproducirse: los topicos no se ven entre dominios DDS, asi que venia del
demonio de ros2cli. La mitigacion pasa de --no-daemon a matarlo.

Se escribe ademas S20_marco_map_prefijado.md, que tres launch citaban desde el
24-ago sin que existiera, y que documenta por que 'map' lleva prefijo. La guia
seguia enseniando lo contrario -"con robot1/map la meta se rechaza"- que es
justo el parrafo que costo una mision abortada.

Tres defectos nuevos quedan anotados en la evidencia, sin arreglar: el vehiculo
sale de la tolerancia estando quieto (93 s sin una sola orden, 4,0 cm), AMCL se
sobreconfia en la aproximacion de frente a la escalera del piso 2, y los siete
controladores compiten entre si al activarse seis en paralelo.
</commit_message>
<xml_diff>
--- a/Documentos/Entregables/Actividad_1_Corte_1_Cronograma_2026-2.xlsx
+++ b/Documentos/Entregables/Actividad_1_Corte_1_Cronograma_2026-2.xlsx
@@ -2339,7 +2339,7 @@
       </c>
       <c r="E16" s="67" t="inlineStr">
         <is>
-          <t>Registro audiovisual y salida de «ros2 node list»; Documentos/Evidencia/S19_dos_agentes.md</t>
+          <t>Documentos/Evidencia/S20_hito_h3_dos_agentes.md, con los dos rosbag2 (/robot1 y /robot2) medidos contra /odom por herramientas/analizar_maniobra.py</t>
         </is>
       </c>
       <c r="F16" s="72" t="inlineStr">
@@ -2362,14 +2362,14 @@
           <t>Réplica del laboratorio en SDF (act. 12) y contrato de interfaces verificado</t>
         </is>
       </c>
-      <c r="J16" s="77" t="inlineStr">
-        <is>
-          <t>En ejecución</t>
+      <c r="J16" s="73" t="inlineStr">
+        <is>
+          <t>Finalizada</t>
         </is>
       </c>
       <c r="K16" s="67" t="inlineStr">
         <is>
-          <t>Hito H3. Los dos agentes ya arrancan aislados con herramientas/robot.sh, cada uno con su dominio ROS y su GAZEBO_MASTER_URI, y cada uno navega sobre el mapa de su nivel: robot1 el 2026-08-21 y robot2 el 2026-08-24. Falta la corrida con los dos a la vez, que es la condición del hito. Sigue abierto el defecto que la bloquea y que contaminaría OE4: una lectura de /odom reportó el desplazamiento del otro robot, y esa lectura apareció justamente con dos agentes corriendo en simultáneo. El desvío de hasta 18° con angular.z = 0 quedó resuelto el 2026-08-18: era el mismo defecto de conversión de angular.z y no una causa aparte</t>
+          <t>Hito H3 cerrado el 2026-08-25: los dos agentes navegaron a la vez, cada uno en su piso, hasta su punto de transferencia. Error real de llegada contra /odom: 0,281 m en robot1 y 0,143 m en robot2. El control es robot2 solo el 2026-08-24, que dio 0,190 m: con un agente en el otro dominio no empeora. El defecto que bloqueaba el hito queda cerrado con causa y no por no reproducirse: los tópicos no se ven entre dominios DDS, así que el /odom cruzado venía del demonio de ros2cli y no de la publicación bajo espacio de nombres; la mitigación pasa de --no-daemon a matar el demonio. Quedan tres defectos nuevos anotados en la evidencia: el vehículo sale de la tolerancia estando quieto (93 s sin una sola orden y 4,0 cm recorridos), AMCL se sobreconfía en la aproximación de frente a la escalera del piso 2, y la activación de los siete controladores compite consigo misma al arrancar seis en paralelo</t>
         </is>
       </c>
     </row>
@@ -2580,12 +2580,12 @@
       </c>
       <c r="J20" s="77" t="inlineStr">
         <is>
-          <t>En ejecución</t>
+          <t>Finalizada</t>
         </is>
       </c>
       <c r="K20" s="67" t="inlineStr">
         <is>
-          <t>Se escribe ANTES de instrumentar, no después. Su dependencia bloqueante quedó resuelta el 2026-08-20: puntos_interes.yaml define 15 destinos del piso 1, de donde salen los orígenes y destinos de las 30 repeticiones. Falta redactar PROTOCOLO_EXPERIMENTAL.md</t>
+          <t>Se escribe ANTES de instrumentar, no después. Un protocolo redactado después de ver los resultados se acomoda sin querer a lo que salió, y la campaña deja de poder refutar nada: la fecha del archivo en el historial de git es parte de la evidencia. Su dependencia bloqueante quedó resuelta el 2026-08-20, cuando puntos_interes.yaml definió los 15 destinos del piso 1, de donde salen los orígenes y destinos de las 30 repeticiones. Documentos/PROTOCOLO_EXPERIMENTAL.md quedó redactado el 2026-08-22 y es la condición 3 de cierre de S19. Fija además que el éxito se mide contra /odom y no contra el SUCCEEDED de Nav2, tras la corrida del 2026-08-21 en que Nav2 devolvió SUCCEEDED a 0,296 m del destino, por encima de la tolerancia configurada de 0,25 m. Lo que queda de OE4 no es este documento sino la instrumentación, que se construye junto con la coordinación (act. 22) y el relevo (act. 26)</t>
         </is>
       </c>
     </row>
@@ -8198,7 +8198,7 @@
       </c>
       <c r="F3" s="75" t="inlineStr">
         <is>
-          <t>55 %. En simulación: un agente navega de forma autónoma con Nav2 + AMCL sobre un mapa derivado de la geometría del mundo, con deriva de 0,045 m frente a la odometría, opera bajo espacio de nombres y el 2026-08-21 alcanza los tres destinos probados sobre el entorno definitivo. Los dos niveles tienen ya mundo y mapa propios, sellados con paneles sintéticos y verificados sin recortes (2026-08-24), y el segundo agente navega sobre el suyo con 0,190 m de error frente a la odometría. En hardware (spike de S19): el LiDAR real repite la misma pared con 2,8 mm de dispersión; el LiDAR de fábrica del kit —un RPLIDAR A1M8-R5— publica /scan con 360 muestras sobre 360° a 6,80 Hz; y el vehículo se comanda desde ROS 2 sin la interfaz web, con dirección y tracción proporcionales. Falta cerrar la cadena /cmd_vel → servo, que el LiDAR conviva con la pila del vehículo —el lanzador pide rplidar_node y el ejecutable instalado se llama rplidar_composition— y la comunicación entre agentes.</t>
+          <t>55 %. En simulación: un agente navega de forma autónoma con Nav2 + AMCL sobre un mapa derivado de la geometría del mundo, con deriva de 0,045 m frente a la odometría, opera bajo espacio de nombres y el 2026-08-21 alcanza los tres destinos probados sobre el entorno definitivo. Los dos niveles tienen ya mundo y mapa propios, sellados con paneles sintéticos y verificados sin recortes (2026-08-24), y el segundo agente navega sobre el suyo con 0,190 m de error frente a la odometría. El 2026-08-25 los dos navegaron a la vez, cada uno en su piso, hasta su punto de transferencia: 0,281 m y 0,143 m frente a la odometría, sin que la simultaneidad degradara al segundo agente. En hardware (spike de S19): el LiDAR real repite la misma pared con 2,8 mm de dispersión; el LiDAR de fábrica del kit —un RPLIDAR A1M8-R5— publica /scan con 360 muestras sobre 360° a 6,80 Hz; y el vehículo se comanda desde ROS 2 sin la interfaz web, con dirección y tracción proporcionales. Falta cerrar la cadena /cmd_vel → servo, que el LiDAR conviva con la pila del vehículo —el lanzador pide rplidar_node y el ejecutable instalado se llama rplidar_composition— y la comunicación entre agentes.</t>
         </is>
       </c>
     </row>
@@ -8279,7 +8279,7 @@
       </c>
       <c r="F5" s="75" t="inlineStr">
         <is>
-          <t>0 %. No existe instrumentación ni protocolo experimental. La dependencia que lo bloqueaba quedó resuelta el 2026-08-20: puntos_interes.yaml define las 15 localizaciones de interés del piso 1, de donde salen los orígenes y destinos de las 30 repeticiones. El protocolo se escribe en S19 y la instrumentación se construye junto con la coordinación (S20) y el relevo (S21), no al final, para que las campañas de S24 y S25 solo tengan que ejecutarse.</t>
+          <t>10 %. El protocolo experimental está escrito y versionado desde el 2026-08-22 (Documentos/PROTOCOLO_EXPERIMENTAL.md, act. 19 de las diez que componen este objetivo): fija las cuatro métricas, N = 30, los criterios de éxito, el tratamiento de la corrida fallida y el formato de registro, y establece que el éxito se mide contra /odom y no contra el SUCCEEDED de Nav2. Su dependencia quedó resuelta el 2026-08-20: puntos_interes.yaml define las localizaciones de interés de donde salen los orígenes y destinos. NO existe todavía instrumentación, ni una sola corrida registrada, ni conjunto de datos: por eso el avance es del 10 % y no más. La instrumentación se construye junto con la coordinación (S20) y el relevo (S21), no al final, para que las campañas de S24 y S25 solo tengan que ejecutarse. Defecto abierto que hoy sesgaría la tasa de éxito: R12, el verificador de meta cuenta como fallo llegadas que fueron buenas</t>
         </is>
       </c>
     </row>
@@ -8466,7 +8466,7 @@
       </c>
       <c r="E4" s="67" t="inlineStr">
         <is>
-          <t>Registro audiovisual y mapas de los dos niveles</t>
+          <t>Los dos rosbag2 de la corrida simultánea y su medición contra /odom, más los mapas de los dos niveles: Documentos/Evidencia/S20_hito_h3_dos_agentes.md</t>
         </is>
       </c>
       <c r="F4" s="67" t="inlineStr">
@@ -8479,9 +8479,9 @@
           <t>Nodo de coordinación</t>
         </is>
       </c>
-      <c r="H4" s="77" t="inlineStr">
-        <is>
-          <t>En ejecución</t>
+      <c r="H4" s="76" t="inlineStr">
+        <is>
+          <t>Finalizada</t>
         </is>
       </c>
     </row>

</xml_diff>